<commit_message>
docs(quauthz): phase labels + tab colors on XLS
Rename XLS tabs to P0–P5 phase format, color-code by status (green=done,
amber=build next, grey=planned, blue=reference), and add phase/status banners
to each sheet title row.

P0 = DONE (sts-delegate-rs), P1 = BUILD NEXT, P2–P5 = PLANNED.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/v2/requirements/QuAuthz-OAuth21-PQC.xlsx
+++ b/docs/v2/requirements/QuAuthz-OAuth21-PQC.xlsx
@@ -9,31 +9,31 @@
   <sheets>
     <sheet name="00 Revision Log" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="01 Executive Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02 Tier0 STS Foundation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03 Tier1 OAuth21 MVP" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04 Tier2 Production" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05 Tier3 High Security" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06 Tier4 Delegation MCP" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07 Tier5 PQC" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="08 Open Issues Map" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09 Standards Matrix" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10 Use Cases" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11 Competitive Summary" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12 Roadmap" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="P0 — STS DONE (sts-delegate-rs)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="P1 — OAuth 2.1 AS (BUILD NEXT)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="P2 — Production Hardening" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="P3 — High Security" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="P4 — Delegation + MCP" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="P5 — PQC" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bugs — Open Issues" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="RFCs — Standards" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="UCs — Use Cases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Competitive" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Roadmap" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00 Revision Log'!$A$2:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Tier0 STS Foundation'!$A$2:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Tier1 OAuth21 MVP'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Tier2 Production'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 Tier3 High Security'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06 Tier4 Delegation MCP'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07 Tier5 PQC'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08 Open Issues Map'!$A$2:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09 Standards Matrix'!$A$2:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10 Use Cases'!$A$2:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11 Competitive Summary'!$A$2:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12 Roadmap'!$A$2:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'P0 — STS DONE (sts-delegate-rs)'!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'P1 — OAuth 2.1 AS (BUILD NEXT)'!$A$2:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'P2 — Production Hardening'!$A$2:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'P3 — High Security'!$A$2:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'P4 — Delegation + MCP'!$A$2:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'P5 — PQC'!$A$2:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Bugs — Open Issues'!$A$2:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'RFCs — Standards'!$A$2:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UCs — Use Cases'!$A$2:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Competitive'!$A$2:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Roadmap'!$A$2:$H$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +42,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +71,18 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +128,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
+        <bgColor rgb="00DAEEF3"/>
       </patternFill>
     </fill>
   </fills>
@@ -246,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -298,6 +326,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,6 +710,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -758,6 +808,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1591,6 +1642,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2004,6 +2056,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2519,6 +2572,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2893,6 +2947,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3024,9 +3079,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>RFC 8693, 9449, 7523, 9728</t>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>DONE — sts-delegate-rs</t>
         </is>
       </c>
     </row>
@@ -3061,9 +3116,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>RFC 9700, 6749, OIDC Core, 9207</t>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>BUILD NEXT — Phase 1</t>
         </is>
       </c>
     </row>
@@ -3098,9 +3153,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>RFC 7009, 7662, 7591, 8707</t>
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>PLANNED — Phase 2</t>
         </is>
       </c>
     </row>
@@ -3135,9 +3190,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>RFC 9449, 9126, 9101, FAPI 2.0</t>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>PLANNED — Phase 3</t>
         </is>
       </c>
     </row>
@@ -3172,9 +3227,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>RFC 8693, 9068, 9728</t>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>PLANNED — Phase 4</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3264,13 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>FIPS 204 (ML-DSA-65), FIPS 203</t>
-        </is>
-      </c>
-    </row>
+      <c r="G12" s="26" t="inlineStr">
+        <is>
+          <t>PLANNED — Phase 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -3367,6 +3423,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0000B050"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3386,16 +3443,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 0 — STS Foundation (SHIPPED) — 97 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Endpoint</t>
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Phase 0 — STS Foundation (DONE: sts-delegate-rs) — 97 Audited Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: SHIPPED as sts-delegate-rs. 87% RFC conformant. 12 open issues tracked in 'Bugs' tab.
+Curls run against: http://127.0.0.1:8888  |  Start: cd sts-delegate-rs &amp;&amp; cargo run --bin sts-cli -- serve</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -8383,6 +8441,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -8402,16 +8461,18 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 1 — OAuth 2.1 MVP (BUILD FIRST) — 49 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Req ID</t>
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Phase 1 — OAuth 2.1 Authorization Server MVP (BUILD NEXT) — ~49 Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: NOT YET BUILT. These are the requirements for the first AS milestone.
+Delivers: /authorize, auth code + PKCE (S256), /token (authorization_code grant), /userinfo, OIDC Discovery.
+Once built, all curls below run against: http://127.0.0.1:8888</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -10939,6 +11000,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -10958,16 +11020,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 2 — Production Hardening — ~20 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Req ID</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Phase 2 — Production Hardening (PLANNED after Phase 1) — ~20 Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: PLANNED. Depends on Phase 1 shipping first. Includes fixes for all 12 open Phase 0 bugs.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -12126,6 +12188,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -12145,16 +12208,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 3 — High Security — ~15 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Req ID</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Phase 3 — High Security Profile (PLANNED) — ~15 Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: PLANNED. DPoP required by default, PAR (/par), JAR, mTLS.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -13048,6 +13111,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -13067,16 +13131,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 4 — Delegation / MCP — ~12 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Req ID</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Phase 4 — Delegation + MCP (PLANNED) — ~12 Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: PLANNED. Wire RFC 8693 delegation into AS. act.iss fix. may_act via consent. MCP-aware audience policy.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -13805,6 +13869,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -13824,16 +13889,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier 5 — Post-Quantum Cryptography — ~12 Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Req ID</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Phase 5 — PQC Profile (PLANNED) — ~12 Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Status: PLANNED. ML-DSA-65 ID tokens, configurable subject token algs, ML-KEM-768 planning (no decrypt oracle per ADR).</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -14612,6 +14677,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>